<commit_message>
update 3 before 4
</commit_message>
<xml_diff>
--- a/Caspar_etal_2022/elife-77875-supp3-v1.xlsx
+++ b/Caspar_etal_2022/elife-77875-supp3-v1.xlsx
@@ -2455,6 +2455,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82E40D92-D6DC-4A92-AB3C-61F5F4215CC4}">
   <ds:schemaRefs>
@@ -2465,4 +2476,8 @@
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93AEFAEB-48AB-49E4-A6B7-3A3BD8F1BAC0}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E80C1498-4169-4E97-BF4F-A08F746194FD}"/>
 </file>
</xml_diff>

<commit_message>
more old changes and new changes
more old changes and new changes
</commit_message>
<xml_diff>
--- a/Caspar_etal_2022/elife-77875-supp3-v1.xlsx
+++ b/Caspar_etal_2022/elife-77875-supp3-v1.xlsx
@@ -2455,6 +2455,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="8e1efd23-f4ba-42d2-85fd-6a510437bae6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82E40D92-D6DC-4A92-AB3C-61F5F4215CC4}">
   <ds:schemaRefs>
@@ -2465,4 +2476,8 @@
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93AEFAEB-48AB-49E4-A6B7-3A3BD8F1BAC0}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{49ACCAE5-E075-4971-8B91-8333F7141A54}"/>
 </file>
</xml_diff>